<commit_message>
feat: add SIDM model center with encrypted credentials
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -2,53 +2,54 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R0cb0b35bd1e04e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="Re651b46f38934793"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="R0b02ea32b5a14de1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="Rd87216b402104a76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="R7802dc240cd64a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="Refaf2445ffeb4958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R5342504da56c40e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="Re156417b97054dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R04d39275eeee4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R99b4ad50b4be4849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="Read7d94ee87540a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="Rfe4cfc83ceb8473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Rb5a53b76c2314a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R0f1a1afa1ce64590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R4e265dcd36514b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="R14a137ce6b744c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="R0cba68697fab4da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="Rdb5536bc31784cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R3ccf1483e5f24365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="R97a6aa7bee8641d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="R739a1b07b06d4365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="R8cb1441f1a1e4f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="R775c4d16b145459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="R4a0634119e1943d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="Rde985372dcaf4950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="R9949677f88794ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="R2b93ff3cc8a145ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="Rd491d499c6144705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="R67f9955a06c645a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="Ra335ceafb0b74aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="R3cfefae86b2d4e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="Reac79fcd5ded4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R24cab977614e40f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R6dbba6b81e474b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="Rbf5c6d944bb249b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="Rb0c265540f404de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="R753b4e9b89f24d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R22792290ad944014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="Rb81c7425baa44529"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R1aab355c20af47a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_config" sheetId="41" r:id="R65cdde767a444e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_sync_record" sheetId="42" r:id="R376a46da444e4da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_follow_up_record" sheetId="43" r:id="Ra846c983c3a54944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_business_attachment" sheetId="44" r:id="R068079ddfe3649a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_client" sheetId="45" r:id="R5732d5608a244423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_record" sheetId="46" r:id="Rbbae3a95f22940ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_request" sheetId="47" r:id="R282d2ba55d4748d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R39038a90b9d0440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R1a78e12b72e6458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="Rcc7ed1e8365e4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R87adb1c3ee834991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="R796d43fd1a5f467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R1ae85d14b12b4408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R15772317f96845bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="Rfdf9524495b74a24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R6f75189ad1344837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R8c74a1bbbe6d4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="R9bd4d094b9f94b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R0b5c1348d1d3414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Ra4a1ded0e6c243bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R7d872087494c4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="Rd4331fcb4bd343b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="R0cb8f5a509d1424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="Rb14919ab7b904a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="R7c85f8f4298841f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R8149bd2f99094c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="R99b7d3c3043344ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="R2b244e81f2d44c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="Rbea91790c31b4427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="Rb541d18fec4f4756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="R4a03188abf534a38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="Refacc2811c954b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="R1457783395af4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="Rf001b66db6fb4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="Radffd48e6f934090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="Rb744287d94154537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="R33229072c31145db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="Rf17269ccfbc54194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="R25183039dfb44ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R76fed14eb3bd47dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R48764335fae24c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="R95ffe68ee04f4a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="R3c3879b2e7bd4d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="R0604836052a94c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R7d381a64f60e49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="R1003f3b095a04fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R711c735094fd44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_config" sheetId="41" r:id="R7983c60cdb924f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_sync_record" sheetId="42" r:id="R4602080f5a7141b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_follow_up_record" sheetId="43" r:id="R200d75c9b1844b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_business_attachment" sheetId="44" r:id="R80f3be7e337f4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_client" sheetId="45" r:id="Rf5f1c32756cc4568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_record" sheetId="46" r:id="R1790ea640d0f48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_request" sheetId="47" r:id="Rce208e9d7f7d427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_llm_connection" sheetId="48" r:id="Rfd2313a9bb4f421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2148,7 +2149,7 @@
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </x:numFmts>
-  <x:fonts count="28">
+  <x:fonts count="29">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -2301,6 +2302,10 @@
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="39">
@@ -2814,7 +2819,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -2930,6 +2935,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -8290,10 +8299,24 @@
         <x:v>执行历史和重复请求防护</x:v>
       </x:c>
     </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>模型中心配置、加密密钥、启停及唯一默认模型。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a04f3c53a84033"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fc7f40851914f61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12072,7 +12095,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="11" t="str">
-        <x:v>共汇总 44 张业务及系统表、548 个字段；全部明细 Sheet 统一使用 10 列字段模板。</x:v>
+        <x:v>共汇总 45 张业务及系统表、561 个字段；全部明细 Sheet 统一使用 10 列字段模板。</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -32662,6 +32685,516 @@
         <x:v>updated_by BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
       </x:c>
     </x:row>
+    <x:row r="553">
+      <x:c r="A553" t="n">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="B553" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C553" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D553" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="E553" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="F553" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="G553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I553"/>
+      <x:c r="J553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K553" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="L553"/>
+      <x:c r="M553" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="N553" t="str">
+        <x:v>BIGSERIAL PRIMARY KEY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554">
+      <x:c r="A554" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="B554" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C554" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D554" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="E554" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="F554" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G554" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H554" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I554"/>
+      <x:c r="J554" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K554"/>
+      <x:c r="L554"/>
+      <x:c r="M554" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="N554" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555">
+      <x:c r="A555" t="n">
+        <x:v>551</x:v>
+      </x:c>
+      <x:c r="B555" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C555" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D555" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="E555" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="F555" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G555" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H555" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I555"/>
+      <x:c r="J555" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K555"/>
+      <x:c r="L555"/>
+      <x:c r="M555" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="N555" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556">
+      <x:c r="A556" t="n">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="B556" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C556" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D556" t="str">
+        <x:v>服务地址</x:v>
+      </x:c>
+      <x:c r="E556" t="str">
+        <x:v>base_url</x:v>
+      </x:c>
+      <x:c r="F556" t="str">
+        <x:v>VARCHAR(500)</x:v>
+      </x:c>
+      <x:c r="G556" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H556" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I556"/>
+      <x:c r="J556" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K556"/>
+      <x:c r="L556"/>
+      <x:c r="M556" t="str">
+        <x:v>公共HTTPS模型地址</x:v>
+      </x:c>
+      <x:c r="N556" t="str">
+        <x:v>VARCHAR(500) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557">
+      <x:c r="A557" t="n">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="B557" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C557" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D557" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="E557" t="str">
+        <x:v>model_name</x:v>
+      </x:c>
+      <x:c r="F557" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G557" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H557" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I557"/>
+      <x:c r="J557" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K557"/>
+      <x:c r="L557"/>
+      <x:c r="M557" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="N557" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558">
+      <x:c r="A558" t="n">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="B558" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C558" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D558" t="str">
+        <x:v>加密API密钥</x:v>
+      </x:c>
+      <x:c r="E558" t="str">
+        <x:v>api_key_ciphertext</x:v>
+      </x:c>
+      <x:c r="F558" t="str">
+        <x:v>TEXT</x:v>
+      </x:c>
+      <x:c r="G558" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H558" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I558"/>
+      <x:c r="J558" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K558"/>
+      <x:c r="L558"/>
+      <x:c r="M558" t="str">
+        <x:v>AES-256-GCM密文，不回显</x:v>
+      </x:c>
+      <x:c r="N558" t="str">
+        <x:v>TEXT NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559">
+      <x:c r="A559" t="n">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="B559" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C559" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D559" t="str">
+        <x:v>启停状态</x:v>
+      </x:c>
+      <x:c r="E559" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="F559" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="G559" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H559" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I559"/>
+      <x:c r="J559" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K559" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L559"/>
+      <x:c r="M559" t="str">
+        <x:v>启停</x:v>
+      </x:c>
+      <x:c r="N559" t="str">
+        <x:v>SMALLINT NOT NULL DEFAULT 0 CHECK (enabled IN (0,1))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560">
+      <x:c r="A560" t="n">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="B560" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C560" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D560" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="E560" t="str">
+        <x:v>is_default</x:v>
+      </x:c>
+      <x:c r="F560" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="G560" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H560" t="str">
+        <x:v>条件唯一</x:v>
+      </x:c>
+      <x:c r="I560"/>
+      <x:c r="J560" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K560" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L560"/>
+      <x:c r="M560" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="N560" t="str">
+        <x:v>SMALLINT NOT NULL DEFAULT 0 CHECK (is_default IN (0,1))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="561">
+      <x:c r="A561" t="n">
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="B561" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C561" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D561" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="E561" t="str">
+        <x:v>timeout_seconds</x:v>
+      </x:c>
+      <x:c r="F561" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="G561" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H561" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I561"/>
+      <x:c r="J561" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K561" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L561"/>
+      <x:c r="M561" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="N561" t="str">
+        <x:v>INTEGER NOT NULL DEFAULT 30 CHECK (timeout_seconds BETWEEN 5 AND 60)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="562">
+      <x:c r="A562" t="n">
+        <x:v>558</x:v>
+      </x:c>
+      <x:c r="B562" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C562" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D562" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="E562" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="F562" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I562" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K562"/>
+      <x:c r="L562"/>
+      <x:c r="M562" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="N562" t="str">
+        <x:v>BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="563">
+      <x:c r="A563" t="n">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="B563" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C563" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D563" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="E563" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="F563" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I563" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K563"/>
+      <x:c r="L563"/>
+      <x:c r="M563" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="N563" t="str">
+        <x:v>BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="564">
+      <x:c r="A564" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="B564" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C564" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D564" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="E564" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="F564" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G564" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H564" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I564"/>
+      <x:c r="J564" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K564" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L564"/>
+      <x:c r="M564" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="N564" t="str">
+        <x:v>TIMESTAMPTZ NOT NULL DEFAULT NOW()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="565">
+      <x:c r="A565" t="n">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="B565" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C565" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D565" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="E565" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="F565" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G565" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H565" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I565"/>
+      <x:c r="J565" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K565" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L565"/>
+      <x:c r="M565" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="N565" t="str">
+        <x:v>TIMESTAMPTZ NOT NULL DEFAULT NOW()</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -32669,7 +33202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf056c0db44c94b7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163537a016994f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33722,7 +34255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R377e21861c7b44df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c154bb306b049e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34301,7 +34834,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36cfcdeeb51642c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8655a4a42dc04546"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34712,7 +35245,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15068c20fa754939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a26926c06e54abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34999,7 +35532,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bc493d6928a44e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0758afec32614f4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35260,7 +35793,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1dcb41f8634976"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a7b7addc0174b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35573,7 +36106,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4d562066004773"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10d42fd41b73412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38871,7 +39404,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e17be8606d54269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77c6a1ad7b4c4b3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40243,6 +40776,427 @@
       <x:c r="I15" s="29"/>
       <x:c r="J15" s="29" t="str">
         <x:v>创建时间</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>pms_llm_connection（模型接入配置表）</x:v>
+      </x:c>
+      <x:c r="B1" s="47"/>
+      <x:c r="C1" s="47"/>
+      <x:c r="D1" s="47"/>
+      <x:c r="E1" s="47"/>
+      <x:c r="F1" s="47"/>
+      <x:c r="G1" s="47"/>
+      <x:c r="H1" s="47"/>
+      <x:c r="I1" s="47"/>
+      <x:c r="J1" s="47"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>中文字段名</x:v>
+      </x:c>
+      <x:c r="B2" s="47" t="str">
+        <x:v>技术字段名</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>数据类型</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>必填</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>是否唯一</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>关联引用</x:v>
+      </x:c>
+      <x:c r="G2" s="47" t="str">
+        <x:v>是否索引</x:v>
+      </x:c>
+      <x:c r="H2" s="47" t="str">
+        <x:v>默认值</x:v>
+      </x:c>
+      <x:c r="I2" s="47" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+      <x:c r="J2" s="47" t="str">
+        <x:v>字段说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="48" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="B3" s="48" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C3" s="48" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="D3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F3" s="48"/>
+      <x:c r="G3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H3" s="48" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="I3" s="48"/>
+      <x:c r="J3" s="48" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="48" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="B4" s="48" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C4" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D4" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E4" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F4" s="48"/>
+      <x:c r="G4" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H4" s="48"/>
+      <x:c r="I4" s="48"/>
+      <x:c r="J4" s="48" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="48" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="C5" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D5" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F5" s="48"/>
+      <x:c r="G5" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H5" s="48"/>
+      <x:c r="I5" s="48"/>
+      <x:c r="J5" s="48" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="48" t="str">
+        <x:v>服务地址</x:v>
+      </x:c>
+      <x:c r="B6" s="48" t="str">
+        <x:v>base_url</x:v>
+      </x:c>
+      <x:c r="C6" s="48" t="str">
+        <x:v>VARCHAR(500)</x:v>
+      </x:c>
+      <x:c r="D6" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E6" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F6" s="48"/>
+      <x:c r="G6" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H6" s="48"/>
+      <x:c r="I6" s="48"/>
+      <x:c r="J6" s="48" t="str">
+        <x:v>公共HTTPS模型地址</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="48" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="B7" s="48" t="str">
+        <x:v>model_name</x:v>
+      </x:c>
+      <x:c r="C7" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D7" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E7" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F7" s="48"/>
+      <x:c r="G7" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H7" s="48"/>
+      <x:c r="I7" s="48"/>
+      <x:c r="J7" s="48" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="48" t="str">
+        <x:v>加密API密钥</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str">
+        <x:v>api_key_ciphertext</x:v>
+      </x:c>
+      <x:c r="C8" s="48" t="str">
+        <x:v>TEXT</x:v>
+      </x:c>
+      <x:c r="D8" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E8" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F8" s="48"/>
+      <x:c r="G8" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H8" s="48"/>
+      <x:c r="I8" s="48"/>
+      <x:c r="J8" s="48" t="str">
+        <x:v>AES-256-GCM密文，不回显</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="48" t="str">
+        <x:v>启停状态</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="D9" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E9" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F9" s="48"/>
+      <x:c r="G9" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H9" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="48"/>
+      <x:c r="J9" s="48" t="str">
+        <x:v>启停</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="48" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="str">
+        <x:v>is_default</x:v>
+      </x:c>
+      <x:c r="C10" s="48" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="D10" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E10" s="48" t="str">
+        <x:v>条件唯一</x:v>
+      </x:c>
+      <x:c r="F10" s="48"/>
+      <x:c r="G10" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H10" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="48"/>
+      <x:c r="J10" s="48" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="48" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="str">
+        <x:v>timeout_seconds</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="D11" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E11" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F11" s="48"/>
+      <x:c r="G11" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H11" s="48" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I11" s="48"/>
+      <x:c r="J11" s="48" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="48" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="B12" s="48" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="C12" s="48" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F12" s="48" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H12" s="48"/>
+      <x:c r="I12" s="48"/>
+      <x:c r="J12" s="48" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="48" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="B13" s="48" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="C13" s="48" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F13" s="48" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H13" s="48"/>
+      <x:c r="I13" s="48"/>
+      <x:c r="J13" s="48" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="47" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F14" s="47"/>
+      <x:c r="G14" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H14" s="47" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I14" s="47"/>
+      <x:c r="J14" s="47" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="47" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="B15" s="47" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F15" s="47"/>
+      <x:c r="G15" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H15" s="47" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I15" s="47"/>
+      <x:c r="J15" s="47" t="str">
+        <x:v>更新时间</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add SIDM model center with encrypted credentials (#59)
Co-authored-by: 孙鑫鑫 <sunxinxin@sunxinxindeMacBook-Pro-2.local>
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -2,53 +2,54 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R0cb0b35bd1e04e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="Re651b46f38934793"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="R0b02ea32b5a14de1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="Rd87216b402104a76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="R7802dc240cd64a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="Refaf2445ffeb4958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R5342504da56c40e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="Re156417b97054dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R04d39275eeee4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R99b4ad50b4be4849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="Read7d94ee87540a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="Rfe4cfc83ceb8473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Rb5a53b76c2314a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R0f1a1afa1ce64590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R4e265dcd36514b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="R14a137ce6b744c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="R0cba68697fab4da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="Rdb5536bc31784cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R3ccf1483e5f24365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="R97a6aa7bee8641d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="R739a1b07b06d4365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="R8cb1441f1a1e4f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="R775c4d16b145459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="R4a0634119e1943d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="Rde985372dcaf4950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="R9949677f88794ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="R2b93ff3cc8a145ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="Rd491d499c6144705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="R67f9955a06c645a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="Ra335ceafb0b74aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="R3cfefae86b2d4e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="Reac79fcd5ded4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R24cab977614e40f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R6dbba6b81e474b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="Rbf5c6d944bb249b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="Rb0c265540f404de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="R753b4e9b89f24d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R22792290ad944014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="Rb81c7425baa44529"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R1aab355c20af47a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_config" sheetId="41" r:id="R65cdde767a444e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_sync_record" sheetId="42" r:id="R376a46da444e4da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_follow_up_record" sheetId="43" r:id="Ra846c983c3a54944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_business_attachment" sheetId="44" r:id="R068079ddfe3649a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_client" sheetId="45" r:id="R5732d5608a244423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_record" sheetId="46" r:id="Rbbae3a95f22940ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_request" sheetId="47" r:id="R282d2ba55d4748d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R39038a90b9d0440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R1a78e12b72e6458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="Rcc7ed1e8365e4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R87adb1c3ee834991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="R796d43fd1a5f467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R1ae85d14b12b4408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R15772317f96845bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="Rfdf9524495b74a24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R6f75189ad1344837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R8c74a1bbbe6d4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="R9bd4d094b9f94b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R0b5c1348d1d3414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Ra4a1ded0e6c243bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R7d872087494c4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="Rd4331fcb4bd343b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="R0cb8f5a509d1424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="Rb14919ab7b904a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="R7c85f8f4298841f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R8149bd2f99094c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="R99b7d3c3043344ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="R2b244e81f2d44c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="Rbea91790c31b4427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="Rb541d18fec4f4756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="R4a03188abf534a38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="Refacc2811c954b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="R1457783395af4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="Rf001b66db6fb4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="Radffd48e6f934090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="Rb744287d94154537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="R33229072c31145db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="Rf17269ccfbc54194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="R25183039dfb44ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R76fed14eb3bd47dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R48764335fae24c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="R95ffe68ee04f4a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="R3c3879b2e7bd4d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="R0604836052a94c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R7d381a64f60e49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="R1003f3b095a04fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R711c735094fd44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_config" sheetId="41" r:id="R7983c60cdb924f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_integration_sync_record" sheetId="42" r:id="R4602080f5a7141b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_follow_up_record" sheetId="43" r:id="R200d75c9b1844b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_business_attachment" sheetId="44" r:id="R80f3be7e337f4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_client" sheetId="45" r:id="Rf5f1c32756cc4568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_record" sheetId="46" r:id="R1790ea640d0f48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_open_request" sheetId="47" r:id="Rce208e9d7f7d427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_llm_connection" sheetId="48" r:id="Rfd2313a9bb4f421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2148,7 +2149,7 @@
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </x:numFmts>
-  <x:fonts count="28">
+  <x:fonts count="29">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -2301,6 +2302,10 @@
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="39">
@@ -2814,7 +2819,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -2930,6 +2935,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -8290,10 +8299,24 @@
         <x:v>执行历史和重复请求防护</x:v>
       </x:c>
     </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>模型中心配置、加密密钥、启停及唯一默认模型。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a04f3c53a84033"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fc7f40851914f61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12072,7 +12095,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="11" t="str">
-        <x:v>共汇总 44 张业务及系统表、548 个字段；全部明细 Sheet 统一使用 10 列字段模板。</x:v>
+        <x:v>共汇总 45 张业务及系统表、561 个字段；全部明细 Sheet 统一使用 10 列字段模板。</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -32662,6 +32685,516 @@
         <x:v>updated_by BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
       </x:c>
     </x:row>
+    <x:row r="553">
+      <x:c r="A553" t="n">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="B553" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C553" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D553" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="E553" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="F553" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="G553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I553"/>
+      <x:c r="J553" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K553" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="L553"/>
+      <x:c r="M553" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="N553" t="str">
+        <x:v>BIGSERIAL PRIMARY KEY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554">
+      <x:c r="A554" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="B554" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C554" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D554" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="E554" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="F554" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G554" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H554" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I554"/>
+      <x:c r="J554" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K554"/>
+      <x:c r="L554"/>
+      <x:c r="M554" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="N554" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555">
+      <x:c r="A555" t="n">
+        <x:v>551</x:v>
+      </x:c>
+      <x:c r="B555" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C555" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D555" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="E555" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="F555" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G555" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H555" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I555"/>
+      <x:c r="J555" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K555"/>
+      <x:c r="L555"/>
+      <x:c r="M555" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="N555" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556">
+      <x:c r="A556" t="n">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="B556" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C556" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D556" t="str">
+        <x:v>服务地址</x:v>
+      </x:c>
+      <x:c r="E556" t="str">
+        <x:v>base_url</x:v>
+      </x:c>
+      <x:c r="F556" t="str">
+        <x:v>VARCHAR(500)</x:v>
+      </x:c>
+      <x:c r="G556" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H556" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I556"/>
+      <x:c r="J556" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K556"/>
+      <x:c r="L556"/>
+      <x:c r="M556" t="str">
+        <x:v>公共HTTPS模型地址</x:v>
+      </x:c>
+      <x:c r="N556" t="str">
+        <x:v>VARCHAR(500) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557">
+      <x:c r="A557" t="n">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="B557" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C557" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D557" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="E557" t="str">
+        <x:v>model_name</x:v>
+      </x:c>
+      <x:c r="F557" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="G557" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H557" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I557"/>
+      <x:c r="J557" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K557"/>
+      <x:c r="L557"/>
+      <x:c r="M557" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="N557" t="str">
+        <x:v>VARCHAR(100) NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558">
+      <x:c r="A558" t="n">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="B558" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C558" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D558" t="str">
+        <x:v>加密API密钥</x:v>
+      </x:c>
+      <x:c r="E558" t="str">
+        <x:v>api_key_ciphertext</x:v>
+      </x:c>
+      <x:c r="F558" t="str">
+        <x:v>TEXT</x:v>
+      </x:c>
+      <x:c r="G558" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H558" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I558"/>
+      <x:c r="J558" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K558"/>
+      <x:c r="L558"/>
+      <x:c r="M558" t="str">
+        <x:v>AES-256-GCM密文，不回显</x:v>
+      </x:c>
+      <x:c r="N558" t="str">
+        <x:v>TEXT NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559">
+      <x:c r="A559" t="n">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="B559" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C559" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D559" t="str">
+        <x:v>启停状态</x:v>
+      </x:c>
+      <x:c r="E559" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="F559" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="G559" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H559" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I559"/>
+      <x:c r="J559" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K559" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L559"/>
+      <x:c r="M559" t="str">
+        <x:v>启停</x:v>
+      </x:c>
+      <x:c r="N559" t="str">
+        <x:v>SMALLINT NOT NULL DEFAULT 0 CHECK (enabled IN (0,1))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560">
+      <x:c r="A560" t="n">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="B560" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C560" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D560" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="E560" t="str">
+        <x:v>is_default</x:v>
+      </x:c>
+      <x:c r="F560" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="G560" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H560" t="str">
+        <x:v>条件唯一</x:v>
+      </x:c>
+      <x:c r="I560"/>
+      <x:c r="J560" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K560" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L560"/>
+      <x:c r="M560" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="N560" t="str">
+        <x:v>SMALLINT NOT NULL DEFAULT 0 CHECK (is_default IN (0,1))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="561">
+      <x:c r="A561" t="n">
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="B561" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C561" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D561" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="E561" t="str">
+        <x:v>timeout_seconds</x:v>
+      </x:c>
+      <x:c r="F561" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="G561" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H561" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I561"/>
+      <x:c r="J561" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K561" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L561"/>
+      <x:c r="M561" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="N561" t="str">
+        <x:v>INTEGER NOT NULL DEFAULT 30 CHECK (timeout_seconds BETWEEN 5 AND 60)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="562">
+      <x:c r="A562" t="n">
+        <x:v>558</x:v>
+      </x:c>
+      <x:c r="B562" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C562" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D562" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="E562" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="F562" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I562" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J562" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K562"/>
+      <x:c r="L562"/>
+      <x:c r="M562" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="N562" t="str">
+        <x:v>BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="563">
+      <x:c r="A563" t="n">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="B563" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C563" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D563" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="E563" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="F563" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I563" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J563" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K563"/>
+      <x:c r="L563"/>
+      <x:c r="M563" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="N563" t="str">
+        <x:v>BIGINT REFERENCES pms_user(id) ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="564">
+      <x:c r="A564" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="B564" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C564" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D564" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="E564" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="F564" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G564" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H564" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I564"/>
+      <x:c r="J564" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K564" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L564"/>
+      <x:c r="M564" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="N564" t="str">
+        <x:v>TIMESTAMPTZ NOT NULL DEFAULT NOW()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="565">
+      <x:c r="A565" t="n">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="B565" t="str">
+        <x:v>pms_llm_connection</x:v>
+      </x:c>
+      <x:c r="C565" t="str">
+        <x:v>模型接入配置表</x:v>
+      </x:c>
+      <x:c r="D565" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="E565" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="F565" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G565" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H565" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="I565"/>
+      <x:c r="J565" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K565" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L565"/>
+      <x:c r="M565" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="N565" t="str">
+        <x:v>TIMESTAMPTZ NOT NULL DEFAULT NOW()</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -32669,7 +33202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf056c0db44c94b7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163537a016994f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33722,7 +34255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R377e21861c7b44df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c154bb306b049e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34301,7 +34834,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36cfcdeeb51642c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8655a4a42dc04546"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34712,7 +35245,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15068c20fa754939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a26926c06e54abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34999,7 +35532,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bc493d6928a44e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0758afec32614f4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35260,7 +35793,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1dcb41f8634976"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a7b7addc0174b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35573,7 +36106,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4d562066004773"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10d42fd41b73412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38871,7 +39404,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e17be8606d54269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77c6a1ad7b4c4b3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40243,6 +40776,427 @@
       <x:c r="I15" s="29"/>
       <x:c r="J15" s="29" t="str">
         <x:v>创建时间</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>pms_llm_connection（模型接入配置表）</x:v>
+      </x:c>
+      <x:c r="B1" s="47"/>
+      <x:c r="C1" s="47"/>
+      <x:c r="D1" s="47"/>
+      <x:c r="E1" s="47"/>
+      <x:c r="F1" s="47"/>
+      <x:c r="G1" s="47"/>
+      <x:c r="H1" s="47"/>
+      <x:c r="I1" s="47"/>
+      <x:c r="J1" s="47"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>中文字段名</x:v>
+      </x:c>
+      <x:c r="B2" s="47" t="str">
+        <x:v>技术字段名</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>数据类型</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>必填</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>是否唯一</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>关联引用</x:v>
+      </x:c>
+      <x:c r="G2" s="47" t="str">
+        <x:v>是否索引</x:v>
+      </x:c>
+      <x:c r="H2" s="47" t="str">
+        <x:v>默认值</x:v>
+      </x:c>
+      <x:c r="I2" s="47" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+      <x:c r="J2" s="47" t="str">
+        <x:v>字段说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="48" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="B3" s="48" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C3" s="48" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="D3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F3" s="48"/>
+      <x:c r="G3" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H3" s="48" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="I3" s="48"/>
+      <x:c r="J3" s="48" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="48" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+      <x:c r="B4" s="48" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C4" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D4" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E4" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F4" s="48"/>
+      <x:c r="G4" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H4" s="48"/>
+      <x:c r="I4" s="48"/>
+      <x:c r="J4" s="48" t="str">
+        <x:v>接入名称</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="48" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="C5" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D5" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F5" s="48"/>
+      <x:c r="G5" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H5" s="48"/>
+      <x:c r="I5" s="48"/>
+      <x:c r="J5" s="48" t="str">
+        <x:v>供应商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="48" t="str">
+        <x:v>服务地址</x:v>
+      </x:c>
+      <x:c r="B6" s="48" t="str">
+        <x:v>base_url</x:v>
+      </x:c>
+      <x:c r="C6" s="48" t="str">
+        <x:v>VARCHAR(500)</x:v>
+      </x:c>
+      <x:c r="D6" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E6" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F6" s="48"/>
+      <x:c r="G6" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H6" s="48"/>
+      <x:c r="I6" s="48"/>
+      <x:c r="J6" s="48" t="str">
+        <x:v>公共HTTPS模型地址</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="48" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+      <x:c r="B7" s="48" t="str">
+        <x:v>model_name</x:v>
+      </x:c>
+      <x:c r="C7" s="48" t="str">
+        <x:v>VARCHAR(100)</x:v>
+      </x:c>
+      <x:c r="D7" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E7" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F7" s="48"/>
+      <x:c r="G7" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H7" s="48"/>
+      <x:c r="I7" s="48"/>
+      <x:c r="J7" s="48" t="str">
+        <x:v>模型标识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="48" t="str">
+        <x:v>加密API密钥</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str">
+        <x:v>api_key_ciphertext</x:v>
+      </x:c>
+      <x:c r="C8" s="48" t="str">
+        <x:v>TEXT</x:v>
+      </x:c>
+      <x:c r="D8" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E8" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F8" s="48"/>
+      <x:c r="G8" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H8" s="48"/>
+      <x:c r="I8" s="48"/>
+      <x:c r="J8" s="48" t="str">
+        <x:v>AES-256-GCM密文，不回显</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="48" t="str">
+        <x:v>启停状态</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="D9" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E9" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F9" s="48"/>
+      <x:c r="G9" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H9" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="48"/>
+      <x:c r="J9" s="48" t="str">
+        <x:v>启停</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="48" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="str">
+        <x:v>is_default</x:v>
+      </x:c>
+      <x:c r="C10" s="48" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="D10" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E10" s="48" t="str">
+        <x:v>条件唯一</x:v>
+      </x:c>
+      <x:c r="F10" s="48"/>
+      <x:c r="G10" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H10" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="48"/>
+      <x:c r="J10" s="48" t="str">
+        <x:v>默认模型</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="48" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="str">
+        <x:v>timeout_seconds</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="D11" s="48" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E11" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F11" s="48"/>
+      <x:c r="G11" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H11" s="48" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I11" s="48"/>
+      <x:c r="J11" s="48" t="str">
+        <x:v>请求超时（秒）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="48" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+      <x:c r="B12" s="48" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="C12" s="48" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F12" s="48" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G12" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H12" s="48"/>
+      <x:c r="I12" s="48"/>
+      <x:c r="J12" s="48" t="str">
+        <x:v>创建人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="48" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+      <x:c r="B13" s="48" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="C13" s="48" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F13" s="48" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G13" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H13" s="48"/>
+      <x:c r="I13" s="48"/>
+      <x:c r="J13" s="48" t="str">
+        <x:v>更新人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="47" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F14" s="47"/>
+      <x:c r="G14" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H14" s="47" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I14" s="47"/>
+      <x:c r="J14" s="47" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="47" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="B15" s="47" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F15" s="47"/>
+      <x:c r="G15" s="47" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H15" s="47" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I15" s="47"/>
+      <x:c r="J15" s="47" t="str">
+        <x:v>更新时间</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add SIDM daily tasks and completion analysis
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -9001,7 +9001,7 @@
         </is>
       </c>
     </row>
-    <row r="7" s="10">
+    <row r="7" s="10" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>关联类型</t>
@@ -9029,7 +9029,7 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>关联类型</t>
+          <t>关联类型：1 项目，2 需求，3 日常任务；日常任务的项目、需求均为空。</t>
         </is>
       </c>
     </row>
@@ -26070,7 +26070,7 @@
         </is>
       </c>
     </row>
-    <row r="209" ht="17" customHeight="1" s="10">
+    <row r="209" s="10" ht="48" customHeight="1">
       <c r="A209" s="6" t="n">
         <v>205</v>
       </c>
@@ -26111,7 +26111,7 @@
       <c r="L209" s="6" t="n"/>
       <c r="M209" s="14" t="inlineStr">
         <is>
-          <t>关联类型</t>
+          <t>关联类型：1 项目，2 需求，3 日常任务；日常任务的项目、需求均为空。</t>
         </is>
       </c>
       <c r="N209" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat: add SIDM daily tasks and completion analysis (#62)
* feat: add SIDM daily tasks and completion analysis

* test: align contract fixture with required requirement date

---------

Co-authored-by: 孙鑫鑫 <sunxinxin@sunxinxindeMacBook-Pro-2.local>
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -9001,7 +9001,7 @@
         </is>
       </c>
     </row>
-    <row r="7" s="10">
+    <row r="7" s="10" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>关联类型</t>
@@ -9029,7 +9029,7 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>关联类型</t>
+          <t>关联类型：1 项目，2 需求，3 日常任务；日常任务的项目、需求均为空。</t>
         </is>
       </c>
     </row>
@@ -26070,7 +26070,7 @@
         </is>
       </c>
     </row>
-    <row r="209" ht="17" customHeight="1" s="10">
+    <row r="209" s="10" ht="48" customHeight="1">
       <c r="A209" s="6" t="n">
         <v>205</v>
       </c>
@@ -26111,7 +26111,7 @@
       <c r="L209" s="6" t="n"/>
       <c r="M209" s="14" t="inlineStr">
         <is>
-          <t>关联类型</t>
+          <t>关联类型：1 项目，2 需求，3 日常任务；日常任务的项目、需求均为空。</t>
         </is>
       </c>
       <c r="N209" s="14" t="inlineStr">

</xml_diff>